<commit_message>
os attendance: show approved leave in its own column, not as absence
The server now returns leave_days apart from absent_count. Without a column
for it, a month of approved leave reads 0 worked / 0 absent with nothing
beside it, which looks like missing data rather than an approved absence —
the mistake one layer along from the one being fixed.

The CSV export carries the same split; it had the old single Absences column.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tmp_payroll/Dubai_Sept_payroll_FOR_CYRINE.xlsx
+++ b/tmp_payroll/Dubai_Sept_payroll_FOR_CYRINE.xlsx
@@ -503,7 +503,7 @@
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
@@ -566,7 +566,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="44" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -582,7 +582,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>marked absent without pay — no clock-in</t>
+          <t>marked absent without pay — no clock-in — her annual leave starts 7 Sep, so this is before it</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -598,7 +598,7 @@
       <c r="G5" s="6" t="inlineStr"/>
       <c r="H5" s="6" t="inlineStr"/>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="44" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
@@ -614,7 +614,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>marked absent without pay — no clock-in</t>
+          <t>marked absent without pay — no clock-in — she has two of these, 4 and 13 Sep</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -630,7 +630,7 @@
       <c r="G6" s="6" t="inlineStr"/>
       <c r="H6" s="6" t="inlineStr"/>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row r="7" ht="44" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
@@ -646,7 +646,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>marked absent without pay — no clock-in</t>
+          <t>marked absent without pay — no clock-in — she has two of these, 4 and 13 Sep</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -662,7 +662,7 @@
       <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="6" t="inlineStr"/>
     </row>
-    <row r="8" ht="32" customHeight="1">
+    <row r="8" ht="44" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
@@ -694,7 +694,7 @@
       <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr"/>
     </row>
-    <row r="9" ht="32" customHeight="1">
+    <row r="9" ht="44" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
@@ -726,7 +726,7 @@
       <c r="G9" s="6" t="inlineStr"/>
       <c r="H9" s="6" t="inlineStr"/>
     </row>
-    <row r="10" ht="32" customHeight="1">
+    <row r="10" ht="44" customHeight="1">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
@@ -758,7 +758,7 @@
       <c r="G10" s="6" t="inlineStr"/>
       <c r="H10" s="6" t="inlineStr"/>
     </row>
-    <row r="11" ht="32" customHeight="1">
+    <row r="11" ht="44" customHeight="1">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
@@ -790,7 +790,7 @@
       <c r="G11" s="6" t="inlineStr"/>
       <c r="H11" s="6" t="inlineStr"/>
     </row>
-    <row r="12" ht="32" customHeight="1">
+    <row r="12" ht="44" customHeight="1">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
@@ -806,7 +806,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>marked absent without pay — no clock-in</t>
+          <t>marked absent without pay — no clock-in — this is his first day back, his annual leave ended 23 Sep. Was the leave extended?</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -822,7 +822,7 @@
       <c r="G12" s="6" t="inlineStr"/>
       <c r="H12" s="6" t="inlineStr"/>
     </row>
-    <row r="13" ht="32" customHeight="1">
+    <row r="13" ht="44" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
@@ -838,7 +838,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>marked absent without pay — no clock-in</t>
+          <t>marked absent without pay — no clock-in — you corrected 15 Sep on the last file; please check whether 14 Sep is the day you meant</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -854,7 +854,7 @@
       <c r="G13" s="6" t="inlineStr"/>
       <c r="H13" s="6" t="inlineStr"/>
     </row>
-    <row r="14" ht="32" customHeight="1">
+    <row r="14" ht="44" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
@@ -886,7 +886,7 @@
       <c r="G14" s="6" t="inlineStr"/>
       <c r="H14" s="6" t="inlineStr"/>
     </row>
-    <row r="15" ht="32" customHeight="1">
+    <row r="15" ht="44" customHeight="1">
       <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
@@ -1708,22 +1708,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Do this on the night of 25 September, before the payroll is computed</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="112" customHeight="1">
+          <t>Run the sync before the payroll is computed — in that order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="144" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>1. Wait until the last shift of 25 September has finished and everyone has clocked out.   2. Run 'Sync from OS Attendance' for Dubai.   3. Then recompute.   Why: 27 people below still had no clock-out for 25 September when this file was made. Computing after 25 September without a re-sync charges each of them a one-hour admin fee for a day that was simply still in progress. The stored figures were also computed on 24 September, before your corrections, so a recompute is needed either way.</t>
+          <t>1. Run 'Sync from OS Attendance' for Dubai.   2. Then recompute.   There is no rush on the clock: 25 September's shifts run late into the evening in Dubai and the clock-outs arrive overnight, so doing this whenever you next pick the payroll up is fine. What matters is only that the sync happens first. Why: when this file was made, the 27 people below had not clocked out for 25 September yet, because they were still at work. The sync is what brings those clock-outs into the DTR. Computing without it charges each of them a one-hour admin fee for a punch that had simply not happened yet. The stored figures also date from 24 September, before your corrections, so a recompute is needed anyway.</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Clocked out now?</t>
+          <t>Clocked out after the sync?</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr"/>

</xml_diff>